<commit_message>
Harden hypothesis mapping retries and extend Vote research outputs.
Per-pass LLM retry stops empty-content failures from aborting dual-run
consensus; add battery/charging schema columns, key_spec-aware projection
trimming, and quadrant map CLI/GUI integration.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/category_templates/phone.xlsx
+++ b/category_templates/phone.xlsx
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -871,22 +871,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>防水和防护</t>
+          <t>电池容量</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>防水和防护</t>
+          <t>电池容量</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>IP等级与机身防护</t>
+          <t>电池额定容量，单位 mAh</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -906,17 +906,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>IP68</t>
+          <t>5000mAh</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>防水;IP68;防护</t>
+          <t>电池;容量;mAh</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>ip_rating</t>
+          <t>mah</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -930,22 +930,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>核心算力与存储</t>
+          <t>充电功率</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>核心算力与存储</t>
+          <t>充电功率</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SoC/GPU/RAM/ROM</t>
+          <t>有线/无线快充功率，单位 W</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>string</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -965,17 +965,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>骁龙8 Gen3；12GB+256GB</t>
+          <t>100W</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>处理器;内存;存储</t>
+          <t>快充;充电功率;瓦</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>storage_combo</t>
+          <t>watt</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -989,17 +989,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>前沿通信能力</t>
+          <t>防水和防护</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>前沿通信能力</t>
+          <t>防水和防护</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5G/Wi-Fi/蓝牙/NFC等</t>
+          <t>IP等级与机身防护</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1019,20 +1019,24 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>5G；Wi-Fi 7；蓝牙5.4；NFC</t>
+          <t>IP68</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>5G;Wi-Fi;蓝牙;NFC</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+          <t>防水;IP68;防护</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ip_rating</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
           <t>multi_claim</t>
@@ -1044,17 +1048,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>屏幕显示技术</t>
+          <t>核心算力与存储</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>屏幕显示技术</t>
+          <t>核心算力与存储</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>尺寸/分辨率/刷新率/亮度</t>
+          <t>SoC/GPU/RAM/ROM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1079,17 +1083,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>6.8英寸 OLED 120Hz</t>
+          <t>骁龙8 Gen3；12GB+256GB</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>屏幕;刷新率;亮度</t>
+          <t>处理器;内存;存储</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>screen_token</t>
+          <t>storage_combo</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1103,17 +1107,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>功耗与续航管理</t>
+          <t>前沿通信能力</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>功耗与续航管理</t>
+          <t>前沿通信能力</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>电池mAh与充电W</t>
+          <t>5G/Wi-Fi/蓝牙/NFC等</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1133,24 +1137,20 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>5000mAh；100W</t>
+          <t>5G；Wi-Fi 7；蓝牙5.4；NFC</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>电池;续航;快充</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>mah;watt</t>
-        </is>
-      </c>
+          <t>5G;Wi-Fi;蓝牙;NFC</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>multi_claim</t>
@@ -1162,17 +1162,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>声学与音频</t>
+          <t>屏幕显示技术</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>声学与音频</t>
+          <t>屏幕显示技术</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>扬声器/麦克风/音频格式</t>
+          <t>尺寸/分辨率/刷新率/亮度</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1192,20 +1192,24 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>立体声双扬声器</t>
+          <t>6.8英寸 OLED 120Hz</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>扬声器;音频</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+          <t>屏幕;刷新率;亮度</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>screen_token</t>
+        </is>
+      </c>
       <c r="K11" t="inlineStr">
         <is>
           <t>multi_claim</t>
@@ -1217,17 +1221,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>智能传感与交互</t>
+          <t>功耗与续航管理</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>智能传感与交互</t>
+          <t>功耗与续航管理</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>指纹/传感器/交互</t>
+          <t>续航叙事与综合功耗描述（容量与功率以专用列为准）</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1252,15 +1256,19 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>屏下指纹；陀螺仪</t>
+          <t>长续航；AI 动态功耗</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>指纹;传感器</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
+          <t>电池;续航;快充</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>mah;watt</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>multi_claim</t>
@@ -1272,17 +1280,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AI底层能力</t>
+          <t>声学与音频</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AI底层能力</t>
+          <t>声学与音频</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>端侧AI/大模型/更新承诺</t>
+          <t>扬声器/麦克风/音频格式</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1307,12 +1315,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>端侧大模型；四年系统更新</t>
+          <t>立体声双扬声器</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>AI;大模型</t>
+          <t>扬声器;音频</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1327,17 +1335,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>核心宣发亮点与差异化功能</t>
+          <t>智能传感与交互</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>核心宣发亮点与差异化功能</t>
+          <t>智能传感与交互</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>发布会主打卖点</t>
+          <t>指纹/传感器/交互</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1362,12 +1370,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>潜望长焦；卫星通信</t>
+          <t>屏下指纹；陀螺仪</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>亮点;卖点</t>
+          <t>指纹;传感器</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1378,6 +1386,116 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AI底层能力</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AI底层能力</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>端侧AI/大模型/更新承诺</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>端侧大模型；四年系统更新</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>AI;大模型</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>multi_claim</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>核心宣发亮点与差异化功能</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>核心宣发亮点与差异化功能</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>发布会主打卖点</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>潜望长焦；卫星通信</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>亮点;卖点</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>multi_claim</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1390,7 +1508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1518,12 +1636,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>防水和防护</t>
+          <t>电池容量</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>防水和防护</t>
+          <t>电池容量</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -1541,12 +1659,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>核心算力与存储</t>
+          <t>充电功率</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>核心算力与存储</t>
+          <t>充电功率</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -1564,12 +1682,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>前沿通信能力</t>
+          <t>防水和防护</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>前沿通信能力</t>
+          <t>防水和防护</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1587,12 +1705,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>屏幕显示技术</t>
+          <t>核心算力与存储</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>屏幕显示技术</t>
+          <t>核心算力与存储</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1610,12 +1728,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>功耗与续航管理</t>
+          <t>前沿通信能力</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>功耗与续航管理</t>
+          <t>前沿通信能力</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1633,12 +1751,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>声学与音频</t>
+          <t>屏幕显示技术</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>声学与音频</t>
+          <t>屏幕显示技术</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1656,12 +1774,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>智能传感与交互</t>
+          <t>功耗与续航管理</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>智能传感与交互</t>
+          <t>功耗与续航管理</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -1679,12 +1797,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>AI底层能力</t>
+          <t>声学与音频</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AI底层能力</t>
+          <t>声学与音频</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1702,18 +1820,64 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>核心宣发亮点与差异化功能</t>
+          <t>智能传感与交互</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>核心宣发亮点与差异化功能</t>
+          <t>智能传感与交互</t>
         </is>
       </c>
       <c r="D14" t="n">
         <v>40</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AI底层能力</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AI底层能力</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>核心宣发亮点与差异化功能</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>核心宣发亮点与差异化功能</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>true</t>
         </is>

</xml_diff>